<commit_message>
used: PDF reader and finish LPs
</commit_message>
<xml_diff>
--- a/Open-LPs - deitado.xlsx
+++ b/Open-LPs - deitado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54FC89BB-F10D-487D-A113-992DF4116799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8ACC98-0763-49F2-A8A3-D7FE5D1DB96B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,279 +20,300 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t>LP</t>
   </si>
   <si>
-    <t>LP-047084</t>
-  </si>
-  <si>
-    <t>LP-047280</t>
-  </si>
-  <si>
-    <t>LP-047413</t>
-  </si>
-  <si>
-    <t>LP-047414</t>
-  </si>
-  <si>
-    <t>LP-047966</t>
-  </si>
-  <si>
-    <t>LP-047967</t>
-  </si>
-  <si>
-    <t>LP-047969</t>
-  </si>
-  <si>
-    <t>LP-047973</t>
-  </si>
-  <si>
-    <t>LP-047974</t>
-  </si>
-  <si>
-    <t>LP-048027</t>
-  </si>
-  <si>
-    <t>LP-048041</t>
-  </si>
-  <si>
-    <t>LP-048076</t>
-  </si>
-  <si>
-    <t>LP-048239</t>
-  </si>
-  <si>
-    <t>LP-048319</t>
-  </si>
-  <si>
-    <t>LP-048525</t>
-  </si>
-  <si>
-    <t>LP-048546</t>
-  </si>
-  <si>
-    <t>LP-048576</t>
-  </si>
-  <si>
-    <t>LP-048591</t>
-  </si>
-  <si>
-    <t>LP-048593</t>
-  </si>
-  <si>
-    <t>LP-048594</t>
-  </si>
-  <si>
-    <t>LP-048595</t>
-  </si>
-  <si>
-    <t>LP-048596</t>
-  </si>
-  <si>
-    <t>LP-048645</t>
-  </si>
-  <si>
-    <t>LP-048655</t>
-  </si>
-  <si>
-    <t>LP-048712</t>
-  </si>
-  <si>
-    <t>LP-048859</t>
-  </si>
-  <si>
-    <t>LP-048902</t>
-  </si>
-  <si>
-    <t>LP-049062</t>
-  </si>
-  <si>
-    <t>LP-049063</t>
-  </si>
-  <si>
-    <t>LP-049064</t>
-  </si>
-  <si>
-    <t>LP-049065</t>
-  </si>
-  <si>
-    <t>LP-049066</t>
-  </si>
-  <si>
-    <t>LP-049068</t>
-  </si>
-  <si>
-    <t>LP-049069</t>
-  </si>
-  <si>
-    <t>LP-049070</t>
-  </si>
-  <si>
-    <t>LP-049072</t>
-  </si>
-  <si>
-    <t>LP-049079</t>
-  </si>
-  <si>
-    <t>LP-049082</t>
-  </si>
-  <si>
-    <t>LP-049084</t>
-  </si>
-  <si>
-    <t>LP-049088</t>
-  </si>
-  <si>
-    <t>LP-049090</t>
-  </si>
-  <si>
-    <t>LP-049113</t>
-  </si>
-  <si>
-    <t>LP-049245</t>
-  </si>
-  <si>
-    <t>LP-049301</t>
-  </si>
-  <si>
-    <t>LP-049302</t>
-  </si>
-  <si>
-    <t>LP-049303</t>
-  </si>
-  <si>
-    <t>LP-049496</t>
-  </si>
-  <si>
-    <t>LP-049498</t>
-  </si>
-  <si>
-    <t>LP-049775</t>
-  </si>
-  <si>
-    <t>LP-049778</t>
-  </si>
-  <si>
-    <t>LP-049817</t>
-  </si>
-  <si>
-    <t>LP-049886</t>
-  </si>
-  <si>
-    <t>LP-049894</t>
-  </si>
-  <si>
-    <t>LP-049916</t>
-  </si>
-  <si>
-    <t>LP-049988</t>
+    <t>LP-041331</t>
+  </si>
+  <si>
+    <t>LP-045379</t>
+  </si>
+  <si>
+    <t>LP-046208</t>
+  </si>
+  <si>
+    <t>LP-046856</t>
+  </si>
+  <si>
+    <t>LP-046871</t>
+  </si>
+  <si>
+    <t>LP-047546</t>
+  </si>
+  <si>
+    <t>LP-047961</t>
+  </si>
+  <si>
+    <t>LP-047994</t>
+  </si>
+  <si>
+    <t>LP-048234</t>
+  </si>
+  <si>
+    <t>LP-048235</t>
+  </si>
+  <si>
+    <t>LP-048237</t>
+  </si>
+  <si>
+    <t>LP-048358</t>
+  </si>
+  <si>
+    <t>LP-048475</t>
+  </si>
+  <si>
+    <t>LP-048483</t>
+  </si>
+  <si>
+    <t>LP-048667</t>
+  </si>
+  <si>
+    <t>LP-048669</t>
+  </si>
+  <si>
+    <t>LP-048689</t>
+  </si>
+  <si>
+    <t>LP-048876</t>
+  </si>
+  <si>
+    <t>LP-048900</t>
+  </si>
+  <si>
+    <t>LP-048977</t>
+  </si>
+  <si>
+    <t>LP-049054</t>
+  </si>
+  <si>
+    <t>LP-049089</t>
+  </si>
+  <si>
+    <t>LP-049144</t>
+  </si>
+  <si>
+    <t>LP-049279</t>
+  </si>
+  <si>
+    <t>LP-049405</t>
+  </si>
+  <si>
+    <t>LP-049408</t>
+  </si>
+  <si>
+    <t>LP-049681</t>
+  </si>
+  <si>
+    <t>LP-049697</t>
+  </si>
+  <si>
+    <t>LP-049698</t>
+  </si>
+  <si>
+    <t>LP-049718</t>
+  </si>
+  <si>
+    <t>LP-049721</t>
+  </si>
+  <si>
+    <t>LP-049722</t>
+  </si>
+  <si>
+    <t>LP-049797</t>
+  </si>
+  <si>
+    <t>LP-049803</t>
+  </si>
+  <si>
+    <t>LP-049804</t>
+  </si>
+  <si>
+    <t>LP-049865</t>
+  </si>
+  <si>
+    <t>LP-049820</t>
+  </si>
+  <si>
+    <t>LP-049867</t>
+  </si>
+  <si>
+    <t>LP-049876</t>
+  </si>
+  <si>
+    <t>LP-049878</t>
+  </si>
+  <si>
+    <t>LP-049879</t>
+  </si>
+  <si>
+    <t>LP-049905</t>
+  </si>
+  <si>
+    <t>LP-049924</t>
+  </si>
+  <si>
+    <t>LP-049941</t>
+  </si>
+  <si>
+    <t>LP-050036</t>
   </si>
   <si>
     <t>LP-050063</t>
   </si>
   <si>
-    <t>LP-050076</t>
-  </si>
-  <si>
-    <t>LP-050677</t>
-  </si>
-  <si>
-    <t>LP-050078</t>
-  </si>
-  <si>
-    <t>LP-050079</t>
-  </si>
-  <si>
-    <t>LP-050080</t>
-  </si>
-  <si>
-    <t>LP-050178</t>
-  </si>
-  <si>
-    <t>LP-050201</t>
-  </si>
-  <si>
-    <t>LP-050321</t>
-  </si>
-  <si>
-    <t>LP-050495</t>
-  </si>
-  <si>
-    <t>LP-050497</t>
-  </si>
-  <si>
-    <t>LP-050499</t>
-  </si>
-  <si>
-    <t>LP-050543</t>
-  </si>
-  <si>
-    <t>LP-050638</t>
-  </si>
-  <si>
-    <t>LP-050641</t>
-  </si>
-  <si>
-    <t>LP-050703</t>
-  </si>
-  <si>
-    <t>LP-050807</t>
-  </si>
-  <si>
-    <t>LP-050808</t>
-  </si>
-  <si>
-    <t>LP-050809</t>
-  </si>
-  <si>
-    <t>LP-050810</t>
-  </si>
-  <si>
-    <t>LP-050811</t>
-  </si>
-  <si>
-    <t>LP-050812</t>
-  </si>
-  <si>
-    <t>LP-050846</t>
-  </si>
-  <si>
-    <t>LP-050885</t>
-  </si>
-  <si>
-    <t>LP-050919</t>
-  </si>
-  <si>
-    <t>LP-044259</t>
-  </si>
-  <si>
-    <t>LP-048461</t>
-  </si>
-  <si>
-    <t>LP-048588</t>
-  </si>
-  <si>
-    <t>LP-048657</t>
-  </si>
-  <si>
-    <t>LP-049087</t>
-  </si>
-  <si>
-    <t>LP-049409</t>
-  </si>
-  <si>
-    <t>LP-050081</t>
-  </si>
-  <si>
-    <t>LP-050250</t>
-  </si>
-  <si>
-    <t>LP-050588</t>
-  </si>
-  <si>
-    <t>LP-050704</t>
+    <t>LP-050111</t>
+  </si>
+  <si>
+    <t>LP-050121</t>
+  </si>
+  <si>
+    <t>LP-050122</t>
+  </si>
+  <si>
+    <t>LP-050149</t>
+  </si>
+  <si>
+    <t>LP-050165</t>
+  </si>
+  <si>
+    <t>LP-050214</t>
+  </si>
+  <si>
+    <t>LP-050215</t>
+  </si>
+  <si>
+    <t>LP-050218</t>
+  </si>
+  <si>
+    <t>LP-050219</t>
+  </si>
+  <si>
+    <t>LP-050220</t>
+  </si>
+  <si>
+    <t>LP-050223</t>
+  </si>
+  <si>
+    <t>LP-050225</t>
+  </si>
+  <si>
+    <t>LP-050240</t>
+  </si>
+  <si>
+    <t>LP-050287</t>
+  </si>
+  <si>
+    <t>LP-050293</t>
+  </si>
+  <si>
+    <t>LP-050294</t>
+  </si>
+  <si>
+    <t>LP-050326</t>
+  </si>
+  <si>
+    <t>LP-050327</t>
+  </si>
+  <si>
+    <t>LP-050335</t>
+  </si>
+  <si>
+    <t>LP-050336</t>
+  </si>
+  <si>
+    <t>LP-050352</t>
+  </si>
+  <si>
+    <t>LP-050368</t>
+  </si>
+  <si>
+    <t>LP-050473</t>
+  </si>
+  <si>
+    <t>LP-050500</t>
+  </si>
+  <si>
+    <t>LP-050507</t>
+  </si>
+  <si>
+    <t>LP-050530</t>
+  </si>
+  <si>
+    <t>LP-050531</t>
+  </si>
+  <si>
+    <t>LP-050534</t>
+  </si>
+  <si>
+    <t>LP-050556</t>
+  </si>
+  <si>
+    <t>LP-050557</t>
+  </si>
+  <si>
+    <t>LP-050562</t>
+  </si>
+  <si>
+    <t>LP-050580</t>
+  </si>
+  <si>
+    <t>LP-050596</t>
+  </si>
+  <si>
+    <t>LP-050618</t>
+  </si>
+  <si>
+    <t>LP-050700</t>
+  </si>
+  <si>
+    <t>LP-050702</t>
+  </si>
+  <si>
+    <t>LP-050727</t>
+  </si>
+  <si>
+    <t>LP-050799</t>
+  </si>
+  <si>
+    <t>LP-050800</t>
+  </si>
+  <si>
+    <t>LP-050876</t>
+  </si>
+  <si>
+    <t>LP-050881</t>
+  </si>
+  <si>
+    <t>LP-051058</t>
+  </si>
+  <si>
+    <t>LP-051104</t>
+  </si>
+  <si>
+    <t>LP-051106</t>
+  </si>
+  <si>
+    <t>LP-051188</t>
+  </si>
+  <si>
+    <t>LP-051194</t>
+  </si>
+  <si>
+    <t>LP-045689</t>
+  </si>
+  <si>
+    <t>LP-048446</t>
+  </si>
+  <si>
+    <t>LP-048460</t>
+  </si>
+  <si>
+    <t>LP-048469</t>
+  </si>
+  <si>
+    <t>LP-050587</t>
   </si>
 </sst>
 </file>
@@ -655,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A91"/>
+  <dimension ref="A1:A98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -668,17 +689,17 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
@@ -733,77 +754,77 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>84</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
@@ -883,237 +904,272 @@
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>85</v>
+        <v>40</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>80</v>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
used: pdf reader kw36
</commit_message>
<xml_diff>
--- a/Open-LPs - deitado.xlsx
+++ b/Open-LPs - deitado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06936724-92C5-45B1-B9C7-6E2220ED7651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0844059-5FF2-40C7-8BD1-A311CD41F948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,198 +20,138 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>LP</t>
   </si>
   <si>
-    <t>LP-033510</t>
-  </si>
-  <si>
-    <t>LP-033548</t>
-  </si>
-  <si>
-    <t>LP-042267</t>
-  </si>
-  <si>
-    <t>LP-047420</t>
-  </si>
-  <si>
-    <t>LP-047986</t>
-  </si>
-  <si>
-    <t>LP-048001</t>
-  </si>
-  <si>
-    <t>LP-048002</t>
-  </si>
-  <si>
-    <t>LP-048178</t>
-  </si>
-  <si>
-    <t>LP-048638</t>
-  </si>
-  <si>
-    <t>LP-048663</t>
-  </si>
-  <si>
-    <t>LP-048718</t>
-  </si>
-  <si>
-    <t>LP-049234</t>
-  </si>
-  <si>
-    <t>LP-049371</t>
-  </si>
-  <si>
-    <t>LP-049551</t>
-  </si>
-  <si>
-    <t>LP-049678</t>
-  </si>
-  <si>
-    <t>LP-050030</t>
-  </si>
-  <si>
-    <t>LP-050126</t>
-  </si>
-  <si>
-    <t>LP-050146</t>
-  </si>
-  <si>
-    <t>LP-050150</t>
-  </si>
-  <si>
-    <t>LP-650151</t>
-  </si>
-  <si>
-    <t>LP-050200</t>
-  </si>
-  <si>
-    <t>LP-050272</t>
-  </si>
-  <si>
-    <t>LP-050313</t>
-  </si>
-  <si>
-    <t>LP-050359</t>
-  </si>
-  <si>
-    <t>LP-050418</t>
-  </si>
-  <si>
-    <t>LP-050424</t>
-  </si>
-  <si>
-    <t>LP-050452</t>
-  </si>
-  <si>
-    <t>LP-050494</t>
-  </si>
-  <si>
-    <t>LP-050498</t>
-  </si>
-  <si>
-    <t>LP-050571</t>
-  </si>
-  <si>
-    <t>LP-050598</t>
-  </si>
-  <si>
-    <t>LP-050685</t>
-  </si>
-  <si>
-    <t>LP-050697</t>
-  </si>
-  <si>
-    <t>LP-050325</t>
-  </si>
-  <si>
-    <t>LP-050836</t>
-  </si>
-  <si>
-    <t>LP-050844</t>
-  </si>
-  <si>
-    <t>LP-050926</t>
-  </si>
-  <si>
-    <t>LP-050961</t>
-  </si>
-  <si>
-    <t>LP-050962</t>
-  </si>
-  <si>
-    <t>LP-050993</t>
-  </si>
-  <si>
-    <t>LP-050994</t>
-  </si>
-  <si>
-    <t>LP-050995</t>
-  </si>
-  <si>
-    <t>LP-050996</t>
-  </si>
-  <si>
-    <t>LP-050997</t>
-  </si>
-  <si>
-    <t>LP-050998</t>
-  </si>
-  <si>
-    <t>LP-050999</t>
-  </si>
-  <si>
-    <t>LP-051026</t>
-  </si>
-  <si>
-    <t>LP-051105</t>
-  </si>
-  <si>
-    <t>LP-051107</t>
-  </si>
-  <si>
-    <t>LP-051119</t>
-  </si>
-  <si>
-    <t>LP-051128</t>
-  </si>
-  <si>
-    <t>LP-051129</t>
-  </si>
-  <si>
-    <t>LP-051251</t>
-  </si>
-  <si>
-    <t>LP-051259</t>
-  </si>
-  <si>
-    <t>LP-051350</t>
-  </si>
-  <si>
-    <t>LP-051453</t>
-  </si>
-  <si>
-    <t>LP-051500</t>
-  </si>
-  <si>
-    <t>LP-051537</t>
-  </si>
-  <si>
-    <t>LP-048392</t>
-  </si>
-  <si>
-    <t>LP-050347</t>
-  </si>
-  <si>
-    <t>LP-050370</t>
-  </si>
-  <si>
-    <t>LP-050599</t>
-  </si>
-  <si>
-    <t>LP-050982</t>
+    <t>LP-047255</t>
+  </si>
+  <si>
+    <t>LP-047649</t>
+  </si>
+  <si>
+    <t>LP-048205</t>
+  </si>
+  <si>
+    <t>LP-048206</t>
+  </si>
+  <si>
+    <t>LP-049726</t>
+  </si>
+  <si>
+    <t>LP-050249</t>
+  </si>
+  <si>
+    <t>LP-050405</t>
+  </si>
+  <si>
+    <t>LP-050889</t>
+  </si>
+  <si>
+    <t>LP-050890</t>
+  </si>
+  <si>
+    <t>LP-050891</t>
+  </si>
+  <si>
+    <t>LP-050392</t>
+  </si>
+  <si>
+    <t>LP-050936</t>
+  </si>
+  <si>
+    <t>LP-051091</t>
+  </si>
+  <si>
+    <t>LP-051143</t>
+  </si>
+  <si>
+    <t>LP-051195</t>
+  </si>
+  <si>
+    <t>LP-051232</t>
+  </si>
+  <si>
+    <t>LP-051254</t>
+  </si>
+  <si>
+    <t>LP-051262</t>
+  </si>
+  <si>
+    <t>LP-051275</t>
+  </si>
+  <si>
+    <t>LP-051276</t>
+  </si>
+  <si>
+    <t>LP-051403</t>
+  </si>
+  <si>
+    <t>LP-051459</t>
+  </si>
+  <si>
+    <t>LP-051531</t>
+  </si>
+  <si>
+    <t>LP-051595</t>
+  </si>
+  <si>
+    <t>LP-051596</t>
+  </si>
+  <si>
+    <t>LP-051611</t>
+  </si>
+  <si>
+    <t>LP-051717</t>
+  </si>
+  <si>
+    <t>LP-051760</t>
+  </si>
+  <si>
+    <t>LP-051891</t>
+  </si>
+  <si>
+    <t>LP-051892</t>
+  </si>
+  <si>
+    <t>LP-051917</t>
+  </si>
+  <si>
+    <t>LP-051924</t>
+  </si>
+  <si>
+    <t>LP-051925</t>
+  </si>
+  <si>
+    <t>LP-051927</t>
+  </si>
+  <si>
+    <t>LP-051929</t>
+  </si>
+  <si>
+    <t>LP-052010</t>
+  </si>
+  <si>
+    <t>LP-052022</t>
+  </si>
+  <si>
+    <t>LP-052041</t>
+  </si>
+  <si>
+    <t>LP-052087</t>
+  </si>
+  <si>
+    <t>LP-046386</t>
+  </si>
+  <si>
+    <t>LP-049057</t>
+  </si>
+  <si>
+    <t>LP-050616</t>
+  </si>
+  <si>
+    <t>LP-052042</t>
   </si>
 </sst>
 </file>
@@ -574,7 +514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -587,137 +527,137 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
@@ -757,147 +697,47 @@
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>62</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: lps and oms feeded
</commit_message>
<xml_diff>
--- a/Open-LPs - deitado.xlsx
+++ b/Open-LPs - deitado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0844059-5FF2-40C7-8BD1-A311CD41F948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C2CDC29-B8BF-4D09-8581-0B218FDF7C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,138 +20,174 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
   <si>
     <t>LP</t>
   </si>
   <si>
-    <t>LP-047255</t>
-  </si>
-  <si>
-    <t>LP-047649</t>
-  </si>
-  <si>
-    <t>LP-048205</t>
-  </si>
-  <si>
-    <t>LP-048206</t>
-  </si>
-  <si>
-    <t>LP-049726</t>
-  </si>
-  <si>
-    <t>LP-050249</t>
-  </si>
-  <si>
-    <t>LP-050405</t>
-  </si>
-  <si>
-    <t>LP-050889</t>
-  </si>
-  <si>
-    <t>LP-050890</t>
-  </si>
-  <si>
-    <t>LP-050891</t>
-  </si>
-  <si>
-    <t>LP-050392</t>
-  </si>
-  <si>
-    <t>LP-050936</t>
-  </si>
-  <si>
-    <t>LP-051091</t>
-  </si>
-  <si>
-    <t>LP-051143</t>
-  </si>
-  <si>
-    <t>LP-051195</t>
-  </si>
-  <si>
-    <t>LP-051232</t>
-  </si>
-  <si>
-    <t>LP-051254</t>
-  </si>
-  <si>
-    <t>LP-051262</t>
-  </si>
-  <si>
-    <t>LP-051275</t>
-  </si>
-  <si>
-    <t>LP-051276</t>
-  </si>
-  <si>
-    <t>LP-051403</t>
-  </si>
-  <si>
-    <t>LP-051459</t>
-  </si>
-  <si>
-    <t>LP-051531</t>
-  </si>
-  <si>
-    <t>LP-051595</t>
-  </si>
-  <si>
-    <t>LP-051596</t>
-  </si>
-  <si>
-    <t>LP-051611</t>
-  </si>
-  <si>
-    <t>LP-051717</t>
-  </si>
-  <si>
-    <t>LP-051760</t>
-  </si>
-  <si>
-    <t>LP-051891</t>
-  </si>
-  <si>
-    <t>LP-051892</t>
-  </si>
-  <si>
-    <t>LP-051917</t>
-  </si>
-  <si>
-    <t>LP-051924</t>
-  </si>
-  <si>
-    <t>LP-051925</t>
-  </si>
-  <si>
-    <t>LP-051927</t>
-  </si>
-  <si>
-    <t>LP-051929</t>
-  </si>
-  <si>
-    <t>LP-052010</t>
-  </si>
-  <si>
-    <t>LP-052022</t>
-  </si>
-  <si>
-    <t>LP-052041</t>
-  </si>
-  <si>
-    <t>LP-052087</t>
-  </si>
-  <si>
-    <t>LP-046386</t>
-  </si>
-  <si>
-    <t>LP-049057</t>
-  </si>
-  <si>
-    <t>LP-050616</t>
-  </si>
-  <si>
-    <t>LP-052042</t>
+    <t>LP-044462</t>
+  </si>
+  <si>
+    <t>LP-045222</t>
+  </si>
+  <si>
+    <t>LP-046519</t>
+  </si>
+  <si>
+    <t>LP-047092</t>
+  </si>
+  <si>
+    <t>LP-047257</t>
+  </si>
+  <si>
+    <t>LP-047258</t>
+  </si>
+  <si>
+    <t>LP-047283</t>
+  </si>
+  <si>
+    <t>LP-047287</t>
+  </si>
+  <si>
+    <t>LP-047294</t>
+  </si>
+  <si>
+    <t>LP-047549</t>
+  </si>
+  <si>
+    <t>LP-047778</t>
+  </si>
+  <si>
+    <t>LP-047989</t>
+  </si>
+  <si>
+    <t>LP-047991</t>
+  </si>
+  <si>
+    <t>LP-048010</t>
+  </si>
+  <si>
+    <t>LP-048343</t>
+  </si>
+  <si>
+    <t>LP-048351</t>
+  </si>
+  <si>
+    <t>LP-048397</t>
+  </si>
+  <si>
+    <t>LP-048426</t>
+  </si>
+  <si>
+    <t>LP-050098</t>
+  </si>
+  <si>
+    <t>LP-050137</t>
+  </si>
+  <si>
+    <t>LP-050248</t>
+  </si>
+  <si>
+    <t>LP-050310</t>
+  </si>
+  <si>
+    <t>LP-050445</t>
+  </si>
+  <si>
+    <t>LP-050895</t>
+  </si>
+  <si>
+    <t>LP-051011</t>
+  </si>
+  <si>
+    <t>LP-051095</t>
+  </si>
+  <si>
+    <t>LP-051172</t>
+  </si>
+  <si>
+    <t>LP-051224</t>
+  </si>
+  <si>
+    <t>LP-051318</t>
+  </si>
+  <si>
+    <t>LP-051319</t>
+  </si>
+  <si>
+    <t>LP-051383</t>
+  </si>
+  <si>
+    <t>LP-051436</t>
+  </si>
+  <si>
+    <t>LP-051626</t>
+  </si>
+  <si>
+    <t>LP-051658</t>
+  </si>
+  <si>
+    <t>LP-051663</t>
+  </si>
+  <si>
+    <t>LP-051756</t>
+  </si>
+  <si>
+    <t>LP-051775</t>
+  </si>
+  <si>
+    <t>LP-051938</t>
+  </si>
+  <si>
+    <t>LP-051967</t>
+  </si>
+  <si>
+    <t>LP-052088</t>
+  </si>
+  <si>
+    <t>LP-052110</t>
+  </si>
+  <si>
+    <t>LP-052133</t>
+  </si>
+  <si>
+    <t>LP-052155</t>
+  </si>
+  <si>
+    <t>LP-052192</t>
+  </si>
+  <si>
+    <t>LP-052253</t>
+  </si>
+  <si>
+    <t>LP-052430</t>
+  </si>
+  <si>
+    <t>LP-052465</t>
+  </si>
+  <si>
+    <t>LP-052479</t>
+  </si>
+  <si>
+    <t>LP-052511</t>
+  </si>
+  <si>
+    <t>LP-052512</t>
+  </si>
+  <si>
+    <t>LP-052516</t>
+  </si>
+  <si>
+    <t>LP-052518</t>
+  </si>
+  <si>
+    <t>LP-052537</t>
+  </si>
+  <si>
+    <t>LP-047454</t>
+  </si>
+  <si>
+    <t>LP-049431</t>
   </si>
 </sst>
 </file>
@@ -514,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -527,22 +563,22 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -552,82 +588,82 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
@@ -732,12 +768,77 @@
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>